<commit_message>
LSLS Oct maybe done
</commit_message>
<xml_diff>
--- a/2026_09_A/2026_09_21/LSLS/LSLS_report_2026-09-25.xlsx
+++ b/2026_09_A/2026_09_21/LSLS/LSLS_report_2026-09-25.xlsx
@@ -8,20 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenalee\work\2026_09\2026_09_A\2026_09_21\LSLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEF0142D-9B5C-4B52-BD62-2D413634ABF6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D31A7FD4-AF2F-4A9D-8491-BD41AB4F4603}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19560" windowHeight="12405" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="reduction of salt.sugar" sheetId="1" r:id="rId1"/>
-    <sheet name="Navigation" sheetId="2" r:id="rId2"/>
+    <sheet name="Navigation" sheetId="4" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="54">
   <si>
     <t>少鹽少糖食店 Daily Badge impression by device</t>
   </si>
@@ -99,6 +100,635 @@
   </si>
   <si>
     <t>16:31:34|| or.search.quick| CityID:0;LndID:35336;Page:1;Lang:zh_TW;Ver:7.21.0; sn:hk.QckSearch</t>
+  </si>
+  <si>
+    <t>ipad</t>
+  </si>
+  <si>
+    <t>15:49:08|| view.SR1.Promotion| CityID:0;sr:sr1;promotionId:13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C12%2C13%2C13%2C13%2C13%2C13%2C13;sn:HK.LMS2.35336.tab.-990.1</t>
+  </si>
+  <si>
+    <t>15:49:06|| or.search.adv| LndID:35336;Page:1;savehistory:true;landmarkCategoryId:-990;subKeyId:-990;keyId:35336;CityID:0;Lang:hk;Ver:7.21.0;sr:(null);sn:HK.AdvSearch</t>
+  </si>
+  <si>
+    <t>15:50:49|| or.search.quick| CityID:0;Lang:hk;Ver:7.21.0;sn:HK.QckSearch</t>
+  </si>
+  <si>
+    <t>15:50:51|| view.SR1.Promotion| CityID:0;sr:sr1;promotionId:13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C12%2C13%2C13%2C13%2C13%2C13%2C13;sn:HK.LMS2.35336.tab.-990.1</t>
+  </si>
+  <si>
+    <t>16:31:42|| view.SR1.Promotion| CityID:0;sr:sr1;promotionId:13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C12%2C13%2C13;sn:HK.Search.SR1.1</t>
+  </si>
+  <si>
+    <t>16:31:39|| or.search.layer.search| Page:1;whatwhere:少鹽少糖;savehistory:true;CityID:0;Lang:hk;Ver:7.22.0;sr:qcksearch;sn:HK.search.layer</t>
+  </si>
+  <si>
+    <t>16:31:38|| or.search.layer| CityID:0;Lang:hk;Ver:7.22.0;sn:HK.Search.SR1.1</t>
+  </si>
+  <si>
+    <t>iphone</t>
+  </si>
+  <si>
+    <t>android</t>
+  </si>
+  <si>
+    <r>
+      <t>CityID:0;PromotionId:13,13,13,13,13,13,13,13,13,13,13,13,13,13,13;Sn:https://www.openrice.com/zh/hongkong/l-%E5%B0%91%E9%B9%BD%E5%B0%91%E7%B3%96%E9%A3%9F%E5%BA%97-l</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>35336</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>CityID:0;PromotionId:13,13,13,13,13,13,13,13,13,13,13,13,13,13,13;Sn:https://www.openrice.com/zh/hongkong/l-%E5%B0%91%E9%B9%BD%E5%B0%91%E7%B3%96%E9%A3%9F%E5%BA%97-l</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>35336</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF041E49"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>?sortBy=ORScoreDesc</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>CityID:0;PromotionId:13,13,13,13,13,13,13,13,13,13,13,13,13,13,13;Sn:https://www.openrice.com/zh/hongkong</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>/restaurants/type/%E5%B0%91%E9%B9%BD%E5%B0%91%E7%B3%96%E9%A3%9F%E5%BA%97</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF041E49"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>?sortBy=ORScoreDesc</t>
+    </r>
+  </si>
+  <si>
+    <t>No LndID</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">16:31:34|| </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>or.search.quick</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>| CityID:0;LndID:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B0F0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>35336</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>;Page:1;Lang:zh_TW;Ver:7.21.0; sn:hk.QckSearch</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>11:25:26||</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> or.search.layer.search</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>| CityID:0;geo:22.2915762%2C114.2081518;LndID:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>35336</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>;Page:1;sr:lmsSr1;Lang:zh_TW;Ver:7.20.4; sn:hk.Search.layer</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>16:31:39||</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> or.search.layer.search</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>| Page:1;whatwhere:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>少鹽少糖</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>;savehistory:true;CityID:0;Lang:hk;Ver:7.22.0;sr:qcksearch;sn:HK.search.layer</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">15:50:49|| </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>or.search.quick| CityID:0;Lang:hk;Ver:7.21.0;sn:HK.QckSearch</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">11:26:28|| </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="7"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>or.search.adv</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>| CityID:0;geo:22.2915762%2C114.2081518;LndID:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="7"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>35336</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>;Page:1;sr:lmsSr1;Lang:zh_TW;Ver:7.20.4; sn:hk.AdvSearch</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>11:26:28||</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> view.SR1.Promotion</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>| CityID:0;PromotionID:13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C12%2C13%2C13%2C13%2C13%2C13%2C13;;Lang:zh_TW;Ver:7.20.4; sn:hk.LMS2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>35336</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.tab.-990.1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">15:49:08|| </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>view.SR1.Promotion</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>| CityID:0;sr:sr1;promotionId:13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C12%2C13%2C13%2C13%2C13%2C13%2C13;sn:HK.LMS2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>35336</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.tab.-990.1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">15:49:06|| </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="7"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>or.search.adv</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>| LndID:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="7"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>35336</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>;Page:1;savehistory:true;landmarkCategoryId:-990;subKeyId:-990;keyId:35336;CityID:0;Lang:hk;Ver:7.21.0;sr:(null);sn:HK.AdvSearch</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">16:34:01|| </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="7"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>or.search.adv</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>| LndID:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="7"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>35336</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>;Page:1;savehistory:true;landmarkCategoryId:-990;subKeyId:-990;keyId:35336;CityID:0;Lang:hk;Ver:7.20.5;tracking:ekeywordsuggestions;sr:(null);sn:HK.AdvSearch</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">16:34:02|| </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>view.SR1.Promotion</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>| CityID:0;sr:sr1;promotionId:13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13;sn:HK.LMS2.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>35336</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.tab.-990.1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">11:25:26|| </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>view.SR1.Promotion</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>| CityID:0;PromotionID:13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C12%2C13%2C13%2C13%2C13%2C13%2C13;;Lang:zh_TW;Ver:7.20.4; sn:hk.LMS2.35336.tab.-990.1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>15:50:51||</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> view.SR1.Promotion</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>| CityID:0;sr:sr1;promotionId:13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C12%2C13%2C13%2C13%2C13%2C13%2C13;sn:HK.LMS2.35336.tab.-990.1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">16:31:42|| </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>view.SR1.Promotion</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>| CityID:0;sr:sr1;promotionId:13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C13%2C12%2C13%2C13;sn:HK.Search.SR1.1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>CityID:0;Sr:Biz;SortBy:ORScoreDesc;LandmarkId:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>35336</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>;UiCity:hongkong;Sn:https://www.openrice.com/zh/hongkong/l-%E5%B0%91%E9%B9%BD%E5%B0%91%E7%B3%96%E9%A3%9F%E5%BA%97-</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="7" tint="-0.249977111117893"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>l</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>35336</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -108,7 +738,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -167,13 +797,66 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="9"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B0F0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="7"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="7"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="7" tint="-0.249977111117893"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -195,6 +878,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="0" tint="-0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -235,7 +924,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
@@ -272,10 +961,19 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -295,6 +993,55 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>390750</xdr:colOff>
+      <xdr:row>60</xdr:row>
+      <xdr:rowOff>152661</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8E531F9D-01E0-4D7C-9F3D-DCB458F890DB}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7381875" y="9725025"/>
+          <a:ext cx="1609950" cy="1867161"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
@@ -308,7 +1055,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1AFF0BDF-4332-438F-9993-B2DC0E0EAED4}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -347,10 +1094,10 @@
     <xdr:ext cx="5400528" cy="4134197"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3">
+        <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000004000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{254AF6CC-0626-4F10-BFF3-639F1B24CBA3}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -366,7 +1113,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="666750" y="6105178"/>
+          <a:off x="666750" y="6124228"/>
           <a:ext cx="5400528" cy="4134197"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -389,10 +1136,10 @@
     <xdr:ext cx="6049835" cy="4594589"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Picture 5">
+        <xdr:cNvPr id="4" name="Picture 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000006000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FA4E6AD6-AC7F-41A1-93A6-E97E0D9D294F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -408,7 +1155,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="676275" y="10858500"/>
+          <a:off x="676275" y="10877550"/>
           <a:ext cx="6049835" cy="4594589"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -431,10 +1178,10 @@
     <xdr:ext cx="5886449" cy="4532045"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Picture 6">
+        <xdr:cNvPr id="5" name="Picture 4">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000007000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A9F83A71-9FAD-40D3-9019-E71D35B64ACB}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -450,7 +1197,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6781800" y="10829925"/>
+          <a:off x="6781800" y="10848975"/>
           <a:ext cx="5886449" cy="4532045"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -473,10 +1220,10 @@
     <xdr:ext cx="2204663" cy="4905375"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="Picture 8">
+        <xdr:cNvPr id="6" name="Picture 5">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000009000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7F11DD95-F1B6-4DBE-9783-71E33938CC05}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -492,7 +1239,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="704850" y="16621125"/>
+          <a:off x="704850" y="16649700"/>
           <a:ext cx="2204663" cy="4905375"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -515,10 +1262,10 @@
     <xdr:ext cx="2183624" cy="4858565"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="10" name="Picture 9">
+        <xdr:cNvPr id="7" name="Picture 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-00000A000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2BCADC9E-2DE8-4D77-BC4E-1A36293FD3BD}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -534,7 +1281,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6179326" y="16590149"/>
+          <a:off x="6179326" y="16618724"/>
           <a:ext cx="2183624" cy="4858565"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -562,10 +1309,10 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="Rectangle 2">
+        <xdr:cNvPr id="8" name="Rectangle 7">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{96FA48BE-B116-46AB-9044-824D60AE7D41}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{96E92B29-2DDC-4D1C-A375-D0EBE68810BF}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -630,10 +1377,10 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="11" name="Rectangle 10">
+        <xdr:cNvPr id="9" name="Rectangle 8">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FD17459D-F40E-43CE-AB14-01B641FE2909}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BB4648E2-F010-4991-8E53-EDE2AC0DDBAC}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -698,10 +1445,10 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="12" name="Rectangle 11">
+        <xdr:cNvPr id="10" name="Rectangle 9">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C1D33915-1BD9-4DF7-9AE2-D5A885F8F7EC}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{419E8341-49D8-4C96-9C34-D126314502A9}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -766,10 +1513,10 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="14" name="Rectangle 13">
+        <xdr:cNvPr id="11" name="Rectangle 10">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{26011CE7-D99E-4019-8FE5-63812589B58E}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8199054B-A9F1-4108-A9A2-3117F560F365}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -834,10 +1581,10 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="15" name="Rectangle 14">
+        <xdr:cNvPr id="12" name="Rectangle 11">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{86165857-C647-467F-B08E-BF3A44072A36}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E92D6314-6242-4529-B2CD-C07AA9E9DCC2}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2487,12 +3234,13 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AE119"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{309A0252-DB31-4DD5-90BE-FBB30F627652}">
+  <dimension ref="A1:AE129"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -2746,9 +3494,370 @@
       <c r="AD119" s="19"/>
       <c r="AE119" s="19"/>
     </row>
+    <row r="120" spans="2:31" x14ac:dyDescent="0.25">
+      <c r="B120" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="121" spans="2:31" x14ac:dyDescent="0.25">
+      <c r="B121" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="122" spans="2:31" x14ac:dyDescent="0.25">
+      <c r="B122" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="123" spans="2:31" x14ac:dyDescent="0.25">
+      <c r="L123" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="124" spans="2:31" x14ac:dyDescent="0.25">
+      <c r="L124" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="125" spans="2:31" x14ac:dyDescent="0.25">
+      <c r="L125" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="126" spans="2:31" x14ac:dyDescent="0.25">
+      <c r="B126" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="127" spans="2:31" x14ac:dyDescent="0.25">
+      <c r="B127" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="128" spans="2:31" x14ac:dyDescent="0.25">
+      <c r="B128" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="129" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B129" t="s">
+        <v>33</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26BDE79B-4FBD-403E-B053-C03F6EB5F47E}">
+  <dimension ref="A1:Z25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A1" s="10"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A3" s="10"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="24" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="18" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="C4" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D4" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="C5" s="10"/>
+      <c r="D5" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="19"/>
+      <c r="M5" s="19"/>
+      <c r="N5" s="19"/>
+      <c r="O5" s="19"/>
+      <c r="P5" s="19"/>
+      <c r="Q5" s="19"/>
+      <c r="R5" s="19"/>
+      <c r="S5" s="19"/>
+      <c r="T5" s="19"/>
+      <c r="U5" s="19"/>
+      <c r="V5" s="19"/>
+      <c r="W5" s="19"/>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="C6" s="10"/>
+      <c r="D6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="B7" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="E7" s="19"/>
+      <c r="F7" s="19"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="19"/>
+      <c r="L7" s="19"/>
+      <c r="M7" s="19"/>
+      <c r="N7" s="19"/>
+      <c r="O7" s="19"/>
+      <c r="P7" s="19"/>
+      <c r="Q7" s="19"/>
+      <c r="R7" s="19"/>
+      <c r="S7" s="19"/>
+      <c r="T7" s="19"/>
+      <c r="U7" s="19"/>
+      <c r="V7" s="19"/>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="C8" s="10"/>
+      <c r="D8" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="C9" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="E9" s="19"/>
+      <c r="F9" s="19"/>
+      <c r="G9" s="19"/>
+      <c r="H9" s="19"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="19"/>
+      <c r="K9" s="19"/>
+      <c r="L9" s="19"/>
+      <c r="M9" s="19"/>
+      <c r="N9" s="19"/>
+      <c r="O9" s="19"/>
+      <c r="P9" s="19"/>
+      <c r="Q9" s="19"/>
+      <c r="R9" s="19"/>
+      <c r="S9" s="19"/>
+      <c r="T9" s="19"/>
+      <c r="U9" s="19"/>
+      <c r="W9" s="20"/>
+      <c r="X9" s="20"/>
+      <c r="Z9" s="22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="C10" s="10"/>
+      <c r="D10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="C11" s="10"/>
+      <c r="D11" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="19"/>
+      <c r="J11" s="19"/>
+    </row>
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A15" s="9"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
+      <c r="A16" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+    </row>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A17" s="9"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="20"/>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="C18" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" s="20" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="C19" s="9"/>
+      <c r="D19" s="19" t="s">
+        <v>45</v>
+      </c>
+      <c r="E19" s="19"/>
+      <c r="F19" s="19"/>
+      <c r="G19" s="19"/>
+      <c r="H19" s="19"/>
+      <c r="I19" s="19"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="19"/>
+      <c r="L19" s="19"/>
+      <c r="M19" s="19"/>
+      <c r="N19" s="19"/>
+      <c r="O19" s="19"/>
+      <c r="P19" s="19"/>
+      <c r="Q19" s="19"/>
+      <c r="R19" s="19"/>
+      <c r="S19" s="19"/>
+      <c r="T19" s="19"/>
+      <c r="U19" s="19"/>
+      <c r="V19" s="19"/>
+      <c r="W19" s="19"/>
+      <c r="X19" s="19"/>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="C20" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="D20" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19"/>
+      <c r="H20" s="19"/>
+      <c r="I20" s="19"/>
+      <c r="J20" s="19"/>
+      <c r="K20" s="19"/>
+      <c r="L20" s="19"/>
+      <c r="M20" s="19"/>
+      <c r="N20" s="19"/>
+      <c r="O20" s="19"/>
+      <c r="P20" s="19"/>
+      <c r="Q20" s="19"/>
+      <c r="R20" s="19"/>
+      <c r="S20" s="19"/>
+      <c r="T20" s="19"/>
+      <c r="U20" s="19"/>
+      <c r="V20" s="19"/>
+      <c r="W20" s="19"/>
+      <c r="X20" s="19"/>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="B21" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C21" s="9"/>
+      <c r="D21" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="C22" s="9"/>
+    </row>
+    <row r="23" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="C23" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="D23" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
+      <c r="G23" s="19"/>
+      <c r="H23" s="19"/>
+      <c r="I23" s="19"/>
+      <c r="J23" s="19"/>
+      <c r="K23" s="19"/>
+      <c r="L23" s="19"/>
+      <c r="M23" s="19"/>
+      <c r="N23" s="19"/>
+      <c r="O23" s="19"/>
+      <c r="P23" s="19"/>
+      <c r="Q23" s="19"/>
+      <c r="R23" s="19"/>
+      <c r="S23" s="19"/>
+      <c r="T23" s="19"/>
+      <c r="U23" s="19"/>
+    </row>
+    <row r="24" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="C24" s="9"/>
+      <c r="D24" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="25" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="C25" s="9"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>